<commit_message>
Add KakaoTalk channel task to 황우중 W31 (5->6 tasks)
Expand directive and completion-report sheets to 6 task rows;
add KakaoTalk Channel (business partner) management; rebalance
weights to 100%.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XPtt2MinYXH5T7wMFXyfVt
</commit_message>
<xml_diff>
--- a/out/BRING_주간_황우중_2026-W31.xlsx
+++ b/out/BRING_주간_황우중_2026-W31.xlsx
@@ -1544,7 +1544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K47"/>
+  <dimension ref="B1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" customWidth="1" style="49" min="2" max="2"/>
@@ -1693,9 +1693,9 @@
       </c>
       <c r="C8" s="70" t="inlineStr">
         <is>
-          <t>황우중 담당자는 당분간 온라인 마케팅 채널 운영과 회사 자료 정리를 담당합니다. 담당 채널은 네이버 블로그·숨고·네이버 플레이스·당근이며, 회사 자료는 구글 드라이브를 정리·문서화합니다.
-핵심 기준은 단순히 게시물·서비스를 올리는 것이 아니라, 각 채널에서 문의와 계약이 얼마나 발생했는지를 '숫자'로 남기는 것입니다. 우중 담당자는 게시·정리·기록·분석까지 맡고, 가격 변경·광고 예산/키워드 변경·외부 공개·파일 삭제는 대표 확인 후 진행합니다.
-업무에는 즉시 진행할 것, 첫 주 내 진행할 것, 매주·매일 반복할 것이 섞여 있으므로, 매일 확인 업무(숨고 신규문의·플레이스 광고 정상노출·광고비 과다소진·전화/톡톡/리뷰·당근 채팅·당일 사진/서류 정리)를 먼저 챙긴 뒤 주간 업무를 진행합니다.</t>
+          <t>황우중 담당자는 당분간 온라인 마케팅 채널 운영과 회사 자료 정리를 담당합니다. 담당 채널은 네이버 블로그·숨고·네이버 플레이스·당근·카카오톡 채널(비즈니스 파트너)이며, 회사 자료는 구글 드라이브를 정리·문서화합니다.
+핵심 기준은 단순히 게시물·서비스를 올리는 것이 아니라, 각 채널에서 문의와 계약이 얼마나 발생했는지를 '숫자'로 남기는 것입니다. 우중 담당자는 게시·정리·기록·분석까지 맡고, 가격 변경·광고 예산/키워드 변경·외부 공개·파일 삭제·광고성 메시지 발송은 대표 확인 후 진행합니다.
+업무에는 즉시 진행할 것, 첫 주 내 진행할 것, 매주·매일 반복할 것이 섞여 있으므로, 매일 확인 업무(숨고 신규문의·플레이스 광고 정상노출·광고비 과다소진·전화/톡톡/리뷰·당근/카카오톡 채팅·당일 사진/서류 정리)를 먼저 챙긴 뒤 주간 업무를 진행합니다.</t>
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C9" s="73" t="inlineStr">
         <is>
-          <t>네이버 블로그·숨고·네이버 플레이스·당근 4개 채널을 정상 운영·최신화하고, 채널별 문의·견적·계약을 숫자로 기록·분석하며, 구글 드라이브 자료를 건물별로 정리·문서화하는 것입니다.</t>
+          <t>네이버 블로그·숨고·네이버 플레이스·당근·카카오톡 채널 5개 채널을 정상 운영·최신화하고, 채널별 문의·견적·계약을 숫자로 기록·분석하며, 구글 드라이브 자료를 건물별로 정리·문서화하는 것입니다.</t>
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
@@ -1872,7 +1872,7 @@
       <c r="B19" s="112" t="n"/>
       <c r="C19" s="113" t="inlineStr">
         <is>
-          <t>공통: 각 채널의 문의·견적·계약을 숫자로 기록하고 매주 금요일 성과 보고</t>
+          <t>6. 카카오톡 채널(비즈니스 파트너) 최신화 및 문의·성과 관리</t>
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
@@ -1886,7 +1886,11 @@
     </row>
     <row r="20" ht="39.75" customHeight="1" s="49">
       <c r="B20" s="112" t="n"/>
-      <c r="C20" s="111" t="n"/>
+      <c r="C20" s="111" t="inlineStr">
+        <is>
+          <t>공통: 각 채널의 문의·견적·계약을 숫자로 기록하고 매주 금요일 성과 보고</t>
+        </is>
+      </c>
       <c r="D20" s="41" t="n"/>
       <c r="E20" s="41" t="n"/>
       <c r="F20" s="41" t="n"/>
@@ -1920,8 +1924,8 @@
 · 가격 변경 / 광고 예산·키워드 추가·삭제 변경
 · 외부 공개·공유 (계약서·신분정보·연락처 등)
 · 원본 파일 삭제·수정 (중복 파일도 바로 삭제하지 말고 목록 보고)
-· 부정 리뷰 답변 (사실관계 확인 필요 리뷰는 바로 보고)
-· 플레이스 기본정보가 실제 운영과 다를 때의 수정</t>
+· 부정 리뷰 답변 / 채널 광고성 메시지(친구 대상) 발송
+· 플레이스·카카오톡 기본정보가 실제 운영과 다를 때의 수정</t>
         </is>
       </c>
       <c r="D22" s="41" t="n"/>
@@ -2080,7 +2084,7 @@
         <is>
           <t>① GitHub 블로그 인수인계 자료 전체를 읽고 운영목적·작성기준·금지사항·사진기준·제목/태그/카테고리 기준을 숙지하고, 이해 안 되는 점은 질문 목록으로 정리합니다.
 ② 전체 게시글 목록을 작성하고, 잘못된 분류·낡은 정보·깨진 사진/링크·중복 글을 찾아 [즉시수정 / 추후보완 / 유지 / 비공개·삭제검토]로 분류합니다.
-③ 신규 포스팅 관리표(작성일·발행일·담당자·제목·핵심/보조 키워드·지역·대상고객·사진·링크·상태·조회수·유입검색어·문의여부)를 만들고 진행상태를 통일합니다(주제선정→자료수집→초안→검수→수정→발행→성과확인).
+③ 신규 포스팅 관리표(작성일·발행일·담당자·제목·핵심/보조 키워드·지역·대상고객·사진·링크·상태·조회수·유입검색어·문의여부)를 만들고 진행상태를 통일합니다.
 ④ 매주 발행 글 수·전체/글별 조회수·유입 검색어·문의 발생 글·다음 주 주제를 확인합니다.</t>
         </is>
       </c>
@@ -2108,7 +2112,7 @@
         <v>8</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="29" ht="123" customHeight="1" s="49">
@@ -2127,9 +2131,9 @@
       </c>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>① 등록 서비스 현황을 점검하고 미완료 서비스·빠진 정보를 확인합니다(지역·설명·가격·사진·연락처).
+          <t>① 등록 서비스 현황을 점검하고 미완료 서비스·빠진 정보를 확인합니다.
 ② 미완료 서비스를 서비스명·소개·지역·작업범위·가격(산정방식)·상담절차·견적방식·작업사진·FAQ로 준비해 등록을 완료합니다.
-③ 숨고 문의 관리표(날짜·지역·요청서비스·건물종류·희망일정·예상견적·견적발송·상담·계약여부·계약금액·실패이유·다음연락일)를 만들고 진행상태를 통일합니다(신규→내용확인→견적준비→견적발송→검토→상담→계약/보류·실패).
+③ 숨고 문의 관리표(날짜·지역·요청서비스·건물종류·희망일정·예상견적·견적발송·상담·계약여부·계약금액·실패이유·다음연락일)를 만들고 진행상태를 통일합니다.
 ④ 매주 문의·견적·상담·계약·계약금액·전환율·사용비용·계약 실패 이유를 정리합니다.</t>
         </is>
       </c>
@@ -2157,7 +2161,7 @@
         <v>6</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="30" ht="84" customHeight="1" s="49">
@@ -2179,7 +2183,7 @@
           <t>① 플레이스 기본정보(업체명·주소·연락처·영업시간·서비스·사진·가격·톡톡 등)를 점검합니다(실제 운영과 다르면 수정 전 대표 확인).
 ② 평일 매일 광고 정상 노출·중단·잔액·예산 소진·키워드 비용 쏠림·문의·리뷰를 확인하고, 이상 시 캡처해 즉시 보고합니다.
 ③ 광고 데이터 기록표(주 3회 이상: 광고비·노출·클릭·클릭률·CPC·전화클릭·톡톡·길찾기·저장·문의·견적·계약·계약금액)를 만들고, 문의당 광고비·계약 전환율·계약당 광고비를 계산합니다.
-④ 매주 검색어·키워드 성과(문의·계약으로 이어진 검색어 / 비용만 든 검색어 / 제외 필요 검색어)를 분석하고 문의 유입경로를 확인합니다. 키워드·예산 변경은 분석 보고 후 진행합니다.</t>
+④ 매주 검색어·키워드 성과(문의·계약으로 이어진 검색어 / 비용만 든 검색어 / 제외 필요)를 분석하고 문의 유입경로를 확인합니다. 키워드·예산 변경은 분석 보고 후 진행합니다.</t>
         </is>
       </c>
       <c r="F30" s="47" t="inlineStr">
@@ -2206,7 +2210,7 @@
         <v>8</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="31" ht="90" customHeight="1" s="49">
@@ -2225,9 +2229,9 @@
       </c>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>① 전체 폴더·파일 현황을 파악합니다(폴더 목록·파일 수·건물/고객/계약/견적/보고서/사진·중복·미분류·열리지 않는 파일·개인정보 포함 파일).
+          <t>① 전체 폴더·파일 현황을 파악합니다(폴더 목록·파일 수·중복·미분류·열리지 않는 파일·개인정보 포함 파일).
 ② 건물별 권장 폴더체계와 파일명 규칙 정리안을 먼저 보고해 승인받습니다(실제 이동 전 승인 필수).
-③ 건물별 기본정보 문서를 작성합니다(건물명·주소·규모·고객·연락처·계약상태·서비스·견적/계약금액·작업주기·서류/사진 링크·특이사항 등, 미확인 항목은 '확인 필요' 표기).
+③ 건물별 기본정보 문서를 작성합니다(건물명·주소·규모·고객·연락처·계약상태·서비스·견적/계약금액·작업주기·서류/사진 링크·특이사항 등, 미확인은 '확인 필요' 표기).
 ④ 완료 결과물(전체 파일목록·건물별 자료목록·누락서류·중복·미분류·개인정보 목록·건물 문서·정리 전후 변경내역)을 제출합니다.</t>
         </is>
       </c>
@@ -2255,7 +2259,7 @@
         <v>7</v>
       </c>
       <c r="K31" s="19" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="32" ht="69" customHeight="1" s="49">
@@ -2275,8 +2279,8 @@
       <c r="E32" s="1" t="inlineStr">
         <is>
           <t>① 기본정보(업체명·대표이미지·소개·연락처·영업시간·지역·서비스·가격·링크·오래된 문구)를 점검·최신화합니다.
-② 기존 게시물을 [유지 / 내용수정 / 사진교체 / 재게시 / 숨김·삭제검토]로 분류합니다(현재 미제공 서비스·낡은 가격/연락처·저품질 사진·중복 확인).
-③ 최신 콘텐츠(회사소개·서비스·활동지역·작업 전후 사진·FAQ·상담방법)를 등록하고, 당근 문의 관리표(날짜·지역·요청서비스·요청사항·답변·견적·계약·실패이유·다음연락일)를 작성합니다.
+② 기존 게시물을 [유지 / 내용수정 / 사진교체 / 재게시 / 숨김·삭제검토]로 분류합니다.
+③ 최신 콘텐츠(회사소개·서비스·활동지역·작업 전후 사진·FAQ·상담방법)를 등록하고, 당근 문의 관리표를 작성합니다.
 ④ 매주 게시물 수·게시물/프로필 조회·관심·채팅/전화 문의·견적·계약·반응 좋은 게시물을 확인합니다.</t>
         </is>
       </c>
@@ -2304,93 +2308,125 @@
         <v>5</v>
       </c>
       <c r="K32" s="19" t="n">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="33" ht="69" customHeight="1" s="49">
-      <c r="B33" s="45" t="inlineStr">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1" s="49">
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>카카오톡 채널(비즈니스 파트너) 최신화 및 관리</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>카카오톡 채널(비즈니스 파트너) 기본정보를 최신화하고, 채팅 문의와 성과를 관리합니다.</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>① 채널 기본정보(채널명·프로필/커버·소개·연락처·영업시간·제공 서비스·홈 노출·링크)를 점검·최신화합니다(실제 운영과 다르면 수정 전 대표 확인).
+② 채널 홈 게시(소식)·안내 문구 현황을 확인하고 낡은 가격·연락처·저품질 사진·중복을 정리 대상으로 분류합니다.
+③ 카카오톡 채널 문의(채팅) 관리표(날짜·지역·요청서비스·건물종류·요청사항·답변·견적·계약·계약금액·실패이유·다음연락일)를 만들고 응대 상태를 통일합니다.
+④ 매주 채널 친구 수·유입·채팅 문의·견적·계약·반응을 확인합니다. 친구 대상 광고성 메시지 발송·가격 변경은 대표 확인 후 진행합니다.</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>06_황우중_카카오톡채널_관리_W31_v1.xlsx</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>브링 구글 드라이브</t>
+        </is>
+      </c>
+      <c r="H33" s="107" t="inlineStr">
+        <is>
+          <t>07-31(금) 17:00</t>
+        </is>
+      </c>
+      <c r="I33" s="47" t="inlineStr">
+        <is>
+          <t>보통</t>
+        </is>
+      </c>
+      <c r="J33" s="114" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" s="19" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="34" ht="69" customHeight="1" s="49">
+      <c r="B34" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="C33" s="51" t="n"/>
-      <c r="D33" s="41" t="n"/>
-      <c r="E33" s="41" t="n"/>
-      <c r="F33" s="41" t="n"/>
-      <c r="G33" s="41" t="n"/>
-      <c r="H33" s="41" t="n"/>
-      <c r="I33" s="42" t="n"/>
-      <c r="J33" s="115">
-        <f>SUM(J28:J32)</f>
-        <v/>
-      </c>
-      <c r="K33" s="21">
-        <f>SUM(K28:K32)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="24" customHeight="1" s="49">
-      <c r="B34" s="45" t="inlineStr">
-        <is>
-          <t>발행 검증</t>
-        </is>
-      </c>
-      <c r="C34" s="116">
-        <f>IF(COUNTA(C28:C32)=0,"업무 미입력",IF(COUNTA(E28:E32)&lt;COUNTA(C28:C32),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F32)&lt;COUNTA(C28:C32),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K32)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K32),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
-        <v/>
-      </c>
+      <c r="C34" s="51" t="n"/>
       <c r="D34" s="41" t="n"/>
       <c r="E34" s="41" t="n"/>
       <c r="F34" s="41" t="n"/>
       <c r="G34" s="41" t="n"/>
       <c r="H34" s="41" t="n"/>
-      <c r="I34" s="41" t="n"/>
-      <c r="J34" s="41" t="n"/>
-      <c r="K34" s="42" t="n"/>
-    </row>
-    <row r="35" ht="24" customHeight="1" s="49"/>
+      <c r="I34" s="42" t="n"/>
+      <c r="J34" s="115">
+        <f>SUM(J28:J33)</f>
+        <v/>
+      </c>
+      <c r="K34" s="21">
+        <f>SUM(K28:K33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="24" customHeight="1" s="49">
+      <c r="B35" s="45" t="inlineStr">
+        <is>
+          <t>발행 검증</t>
+        </is>
+      </c>
+      <c r="C35" s="116">
+        <f>IF(COUNTA(C28:C33)=0,"업무 미입력",IF(COUNTA(E28:E33)&lt;COUNTA(C28:C33),"발행 불가 — 완료기준 누락 업무 있음",IF(COUNTA(F28:F33)&lt;COUNTA(C28:C33),"발행 불가 — 산출물 누락 업무 있음",IF(SUM(K28:K33)&lt;&gt;1,"발행 불가 — 가중치 합계 "&amp;TEXT(SUM(K28:K33),"0%")&amp;" (100% 필요)","발행 가능 — 완료기준·산출물·가중치 충족"))))</f>
+        <v/>
+      </c>
+      <c r="D35" s="41" t="n"/>
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="41" t="n"/>
+      <c r="G35" s="41" t="n"/>
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="41" t="n"/>
+      <c r="J35" s="41" t="n"/>
+      <c r="K35" s="42" t="n"/>
+    </row>
     <row r="36" ht="24" customHeight="1" s="49"/>
-    <row r="37" ht="18" customHeight="1" s="49">
-      <c r="B37" s="89" t="inlineStr">
+    <row r="37" ht="24" customHeight="1" s="49">
+      <c r="B37" s="89" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="49">
+      <c r="B38" s="89" t="inlineStr">
         <is>
           <t>담당자 접수확인  —  월요일 12:00까지 담당자 직접 작성 (미작성 = 업무 미이해로 간주, 재지시)</t>
         </is>
       </c>
-      <c r="C37" s="64" t="n"/>
-      <c r="D37" s="64" t="n"/>
-      <c r="E37" s="64" t="n"/>
-      <c r="F37" s="64" t="n"/>
-      <c r="G37" s="64" t="n"/>
-      <c r="H37" s="64" t="n"/>
-      <c r="I37" s="64" t="n"/>
-      <c r="J37" s="64" t="n"/>
-      <c r="K37" s="64" t="n"/>
-    </row>
-    <row r="38" ht="36" customHeight="1" s="49">
-      <c r="B38" s="45" t="inlineStr">
+      <c r="C38" s="64" t="n"/>
+      <c r="D38" s="64" t="n"/>
+      <c r="E38" s="64" t="n"/>
+      <c r="F38" s="64" t="n"/>
+      <c r="G38" s="64" t="n"/>
+      <c r="H38" s="64" t="n"/>
+      <c r="I38" s="64" t="n"/>
+      <c r="J38" s="64" t="n"/>
+      <c r="K38" s="64" t="n"/>
+    </row>
+    <row r="39" ht="36" customHeight="1" s="49">
+      <c r="B39" s="45" t="inlineStr">
         <is>
           <t>내가 이해한 업무
 (본인 언어로 재작성)</t>
         </is>
       </c>
-      <c r="C38" s="117" t="n"/>
-      <c r="D38" s="41" t="n"/>
-      <c r="E38" s="41" t="n"/>
-      <c r="F38" s="41" t="n"/>
-      <c r="G38" s="41" t="n"/>
-      <c r="H38" s="41" t="n"/>
-      <c r="I38" s="41" t="n"/>
-      <c r="J38" s="41" t="n"/>
-      <c r="K38" s="42" t="n"/>
-    </row>
-    <row r="39" ht="19.5" customHeight="1" s="49">
-      <c r="B39" s="45" t="inlineStr">
-        <is>
-          <t>완료기준 재확인
-(무엇이 되면 끝인가)</t>
-        </is>
-      </c>
-      <c r="C39" s="118" t="n"/>
+      <c r="C39" s="117" t="n"/>
       <c r="D39" s="41" t="n"/>
       <c r="E39" s="41" t="n"/>
       <c r="F39" s="41" t="n"/>
@@ -2400,14 +2436,14 @@
       <c r="J39" s="41" t="n"/>
       <c r="K39" s="42" t="n"/>
     </row>
-    <row r="40" ht="24" customHeight="1" s="49">
+    <row r="40" ht="19.5" customHeight="1" s="49">
       <c r="B40" s="45" t="inlineStr">
         <is>
-          <t>예상 리스크
-(막힐 것 같은 지점)</t>
-        </is>
-      </c>
-      <c r="C40" s="43" t="n"/>
+          <t>완료기준 재확인
+(무엇이 되면 끝인가)</t>
+        </is>
+      </c>
+      <c r="C40" s="118" t="n"/>
       <c r="D40" s="41" t="n"/>
       <c r="E40" s="41" t="n"/>
       <c r="F40" s="41" t="n"/>
@@ -2420,7 +2456,8 @@
     <row r="41" ht="24" customHeight="1" s="49">
       <c r="B41" s="45" t="inlineStr">
         <is>
-          <t>필요한 지원·의사결정</t>
+          <t>예상 리스크
+(막힐 것 같은 지점)</t>
         </is>
       </c>
       <c r="C41" s="43" t="n"/>
@@ -2436,7 +2473,7 @@
     <row r="42" ht="24" customHeight="1" s="49">
       <c r="B42" s="45" t="inlineStr">
         <is>
-          <t>실행 계획 (요일 배분)</t>
+          <t>필요한 지원·의사결정</t>
         </is>
       </c>
       <c r="C42" s="43" t="n"/>
@@ -2452,10 +2489,10 @@
     <row r="43" ht="24" customHeight="1" s="49">
       <c r="B43" s="45" t="inlineStr">
         <is>
-          <t>접수 확인 일시 / 서명</t>
-        </is>
-      </c>
-      <c r="C43" s="47" t="n"/>
+          <t>실행 계획 (요일 배분)</t>
+        </is>
+      </c>
+      <c r="C43" s="43" t="n"/>
       <c r="D43" s="41" t="n"/>
       <c r="E43" s="41" t="n"/>
       <c r="F43" s="41" t="n"/>
@@ -2465,96 +2502,113 @@
       <c r="J43" s="41" t="n"/>
       <c r="K43" s="42" t="n"/>
     </row>
-    <row r="44" ht="24" customHeight="1" s="49"/>
+    <row r="44" ht="24" customHeight="1" s="49">
+      <c r="B44" s="45" t="inlineStr">
+        <is>
+          <t>접수 확인 일시 / 서명</t>
+        </is>
+      </c>
+      <c r="C44" s="47" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n"/>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="41" t="n"/>
+      <c r="J44" s="41" t="n"/>
+      <c r="K44" s="42" t="n"/>
+    </row>
     <row r="45" ht="24" customHeight="1" s="49">
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" s="4" t="n"/>
+    </row>
+    <row r="46" ht="24" customHeight="1" s="49">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>결   재</t>
         </is>
       </c>
-      <c r="C45" s="41" t="n"/>
-      <c r="D45" s="41" t="n"/>
-      <c r="E45" s="41" t="n"/>
-      <c r="F45" s="41" t="n"/>
-      <c r="G45" s="41" t="n"/>
-      <c r="H45" s="41" t="n"/>
-      <c r="I45" s="41" t="n"/>
-      <c r="J45" s="41" t="n"/>
-      <c r="K45" s="42" t="n"/>
-    </row>
-    <row r="46" ht="24" customHeight="1" s="49">
-      <c r="B46" s="45" t="inlineStr">
+      <c r="C46" s="41" t="n"/>
+      <c r="D46" s="41" t="n"/>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+      <c r="H46" s="41" t="n"/>
+      <c r="I46" s="41" t="n"/>
+      <c r="J46" s="41" t="n"/>
+      <c r="K46" s="42" t="n"/>
+    </row>
+    <row r="47" ht="24" customHeight="1" s="49">
+      <c r="B47" s="45" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C46" s="45" t="inlineStr">
+      <c r="C47" s="45" t="inlineStr">
         <is>
           <t>작성 (지시자)</t>
         </is>
       </c>
-      <c r="D46" s="42" t="n"/>
-      <c r="E46" s="45" t="inlineStr">
+      <c r="D47" s="42" t="n"/>
+      <c r="E47" s="45" t="inlineStr">
         <is>
           <t>검토 (검수자)</t>
         </is>
       </c>
-      <c r="F46" s="42" t="n"/>
-      <c r="G46" s="45" t="inlineStr">
+      <c r="F47" s="42" t="n"/>
+      <c r="G47" s="45" t="inlineStr">
         <is>
           <t>승인 (대표)</t>
         </is>
       </c>
-      <c r="H46" s="42" t="n"/>
-      <c r="I46" s="45" t="inlineStr">
+      <c r="H47" s="42" t="n"/>
+      <c r="I47" s="45" t="inlineStr">
         <is>
           <t>접수 (담당자)</t>
         </is>
       </c>
-      <c r="J46" s="42" t="n"/>
-      <c r="K46" s="45" t="inlineStr">
+      <c r="J47" s="42" t="n"/>
+      <c r="K47" s="45" t="inlineStr">
         <is>
           <t>일자</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="45" t="inlineStr">
+    <row r="48" ht="19.5" customHeight="1" s="49">
+      <c r="B48" s="45" t="inlineStr">
         <is>
           <t>서명</t>
         </is>
       </c>
-      <c r="C47" s="47" t="inlineStr">
+      <c r="C48" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="D47" s="42" t="n"/>
-      <c r="E47" s="47" t="inlineStr">
+      <c r="D48" s="42" t="n"/>
+      <c r="E48" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="F47" s="42" t="n"/>
-      <c r="G47" s="47" t="inlineStr">
+      <c r="F48" s="42" t="n"/>
+      <c r="G48" s="47" t="inlineStr">
         <is>
           <t>서 창 환</t>
         </is>
       </c>
-      <c r="H47" s="42" t="n"/>
-      <c r="I47" s="47" t="inlineStr">
+      <c r="H48" s="42" t="n"/>
+      <c r="I48" s="47" t="inlineStr">
         <is>
           <t>황 우 중</t>
         </is>
       </c>
-      <c r="J47" s="42" t="n"/>
-      <c r="K47" s="109" t="inlineStr">
+      <c r="J48" s="42" t="n"/>
+      <c r="K48" s="109" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="19.5" customHeight="1" s="49"/>
     <row r="49" ht="21.75" customHeight="1" s="49"/>
     <row r="50" ht="21.75" customHeight="1" s="49"/>
     <row r="51" ht="21.75" customHeight="1" s="49"/>
@@ -2575,48 +2629,48 @@
     <row r="68" ht="39.75" customHeight="1" s="49"/>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="C41:K41"/>
     <mergeCell ref="C10:K10"/>
-    <mergeCell ref="C41:K41"/>
     <mergeCell ref="C15:J15"/>
-    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="C44:K44"/>
     <mergeCell ref="C24:J24"/>
     <mergeCell ref="C40:K40"/>
     <mergeCell ref="C9:K9"/>
     <mergeCell ref="C14:J14"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="G48:H48"/>
     <mergeCell ref="C43:K43"/>
-    <mergeCell ref="B45:K45"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="I47:J47"/>
     <mergeCell ref="C20:J20"/>
     <mergeCell ref="B26:K26"/>
     <mergeCell ref="C16:J16"/>
+    <mergeCell ref="C34:I34"/>
     <mergeCell ref="B7:K7"/>
     <mergeCell ref="C39:K39"/>
+    <mergeCell ref="C22:J22"/>
     <mergeCell ref="C8:K8"/>
-    <mergeCell ref="C22:J22"/>
-    <mergeCell ref="C33:I33"/>
     <mergeCell ref="B14:B21"/>
-    <mergeCell ref="C38:K38"/>
-    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="B46:K46"/>
     <mergeCell ref="C21:J21"/>
-    <mergeCell ref="E46:F46"/>
     <mergeCell ref="B12:K12"/>
     <mergeCell ref="B2:K2"/>
-    <mergeCell ref="C34:K34"/>
+    <mergeCell ref="C48:D48"/>
+    <mergeCell ref="I48:J48"/>
     <mergeCell ref="C23:J23"/>
     <mergeCell ref="C17:J17"/>
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="G47:H47"/>
     <mergeCell ref="C42:K42"/>
-    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="C13:J13"/>
     <mergeCell ref="C19:J19"/>
-    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="C35:K35"/>
+    <mergeCell ref="B38:K38"/>
+    <mergeCell ref="E47:F47"/>
     <mergeCell ref="C18:J18"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="B37:K37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="I28:I32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I28:I33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"최우선,높음,보통,낮음"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2631,7 +2685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C1:L47"/>
+  <dimension ref="C1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="19.85546875" customWidth="1" style="49" min="3" max="3"/>
@@ -2712,7 +2766,7 @@
         </is>
       </c>
       <c r="D5" s="26">
-        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
+        <f>SUMPRODUCT(F12:F17,H12:H17)</f>
         <v/>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2730,7 +2784,7 @@
         </is>
       </c>
       <c r="H5" s="119">
-        <f>SUM('01_업무지시서'!J28:J32)</f>
+        <f>SUM('01_업무지시서'!J28:J33)</f>
         <v/>
       </c>
       <c r="I5" s="4" t="inlineStr">
@@ -2739,7 +2793,7 @@
         </is>
       </c>
       <c r="J5" s="119">
-        <f>SUM(I12:I16)</f>
+        <f>SUM(I12:I17)</f>
         <v/>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -3021,109 +3075,118 @@
       <c r="K16" s="47" t="n"/>
       <c r="L16" s="47" t="n"/>
     </row>
-    <row r="17" ht="15" customHeight="1" s="49">
-      <c r="C17" s="45" t="inlineStr">
+    <row r="17" ht="27.75" customHeight="1" s="49">
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="40">
+        <f>IF('01_업무지시서'!C33="","",'01_업무지시서'!C33)</f>
+        <v/>
+      </c>
+      <c r="E17" s="40">
+        <f>IF('01_업무지시서'!E33="","",'01_업무지시서'!E33)</f>
+        <v/>
+      </c>
+      <c r="F17" s="11">
+        <f>IF('01_업무지시서'!K33="",0,'01_업무지시서'!K33)</f>
+        <v/>
+      </c>
+      <c r="G17" s="47" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="114" t="n"/>
+      <c r="J17" s="47" t="n"/>
+      <c r="K17" s="47" t="n"/>
+      <c r="L17" s="47" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="49">
+      <c r="C18" s="45" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="D17" s="45" t="inlineStr">
+      <c r="D18" s="45" t="inlineStr">
         <is>
           <t>가중 달성률 →</t>
         </is>
       </c>
-      <c r="E17" s="42" t="n"/>
-      <c r="F17" s="21">
-        <f>SUM(F12:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="28">
-        <f>SUMPRODUCT(F12:F16,H12:H16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="29">
-        <f>COUNTIF(G12:G16,"완료")</f>
-        <v/>
-      </c>
-      <c r="I17" s="115">
-        <f>SUM(I12:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="69">
-        <f>"완료 "&amp;COUNTIF(G12:G16,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G16,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G16,"미착수")&amp;"건"</f>
-        <v/>
-      </c>
-      <c r="K17" s="41" t="n"/>
-      <c r="L17" s="42" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1" s="49">
-      <c r="C18" s="46" t="n"/>
-      <c r="D18" s="46" t="n"/>
-      <c r="I18" s="46" t="n"/>
-      <c r="J18" s="46" t="n"/>
-      <c r="L18" s="46" t="n"/>
-    </row>
-    <row r="19" ht="19.5" customHeight="1" s="49">
-      <c r="C19" s="121" t="inlineStr">
+      <c r="E18" s="42" t="n"/>
+      <c r="F18" s="21">
+        <f>SUM(F12:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="28">
+        <f>SUMPRODUCT(F12:F17,H12:H17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="29">
+        <f>COUNTIF(G12:G17,"완료")</f>
+        <v/>
+      </c>
+      <c r="I18" s="115">
+        <f>SUM(I12:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="69">
+        <f>"완료 "&amp;COUNTIF(G12:G17,"완료")&amp;"건 / 진행중 "&amp;COUNTIF(G12:G17,"진행중")&amp;"건 / 미착수 "&amp;COUNTIF(G12:G17,"미착수")&amp;"건"</f>
+        <v/>
+      </c>
+      <c r="K18" s="41" t="n"/>
+      <c r="L18" s="42" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="49">
+      <c r="C19" s="46" t="n"/>
+      <c r="D19" s="46" t="n"/>
+      <c r="I19" s="46" t="n"/>
+      <c r="J19" s="46" t="n"/>
+      <c r="L19" s="46" t="n"/>
+    </row>
+    <row r="20" ht="19.5" customHeight="1" s="49">
+      <c r="C20" s="121" t="inlineStr">
         <is>
           <t>2. 자가 검수  —  제출 전 §4 검수기준으로 본인이 먼저 점검</t>
         </is>
       </c>
-      <c r="D19" s="64" t="n"/>
-      <c r="E19" s="64" t="n"/>
-      <c r="F19" s="64" t="n"/>
-      <c r="G19" s="64" t="n"/>
-      <c r="H19" s="64" t="n"/>
-      <c r="I19" s="64" t="n"/>
-      <c r="J19" s="64" t="n"/>
-      <c r="K19" s="64" t="n"/>
-      <c r="L19" s="65" t="n"/>
-    </row>
-    <row r="20" ht="24" customHeight="1" s="49">
-      <c r="C20" s="46" t="inlineStr">
+      <c r="D20" s="64" t="n"/>
+      <c r="E20" s="64" t="n"/>
+      <c r="F20" s="64" t="n"/>
+      <c r="G20" s="64" t="n"/>
+      <c r="H20" s="64" t="n"/>
+      <c r="I20" s="64" t="n"/>
+      <c r="J20" s="64" t="n"/>
+      <c r="K20" s="64" t="n"/>
+      <c r="L20" s="65" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1" s="49">
+      <c r="C21" s="46" t="inlineStr">
         <is>
           <t>검수 항목 (자동)</t>
         </is>
       </c>
-      <c r="D20" s="46" t="inlineStr">
+      <c r="D21" s="46" t="inlineStr">
         <is>
           <t>검수 질문 (자동)</t>
         </is>
       </c>
-      <c r="E20" s="41" t="n"/>
-      <c r="F20" s="41" t="n"/>
-      <c r="G20" s="41" t="n"/>
-      <c r="H20" s="42" t="n"/>
-      <c r="I20" s="46" t="inlineStr">
-        <is>
-          <t>자가
-판정</t>
-        </is>
-      </c>
-      <c r="J20" s="46" t="inlineStr">
-        <is>
-          <t>미충족 사유·보완 계획</t>
-        </is>
-      </c>
-      <c r="K20" s="42" t="n"/>
-      <c r="L20" s="46" t="inlineStr">
-        <is>
-          <t>검수자
-판정</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1" s="49">
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="55" t="n"/>
       <c r="E21" s="41" t="n"/>
       <c r="F21" s="41" t="n"/>
       <c r="G21" s="41" t="n"/>
       <c r="H21" s="42" t="n"/>
-      <c r="I21" s="47" t="n"/>
-      <c r="J21" s="44" t="n"/>
+      <c r="I21" s="46" t="inlineStr">
+        <is>
+          <t>자가
+판정</t>
+        </is>
+      </c>
+      <c r="J21" s="46" t="inlineStr">
+        <is>
+          <t>미충족 사유·보완 계획</t>
+        </is>
+      </c>
       <c r="K21" s="42" t="n"/>
-      <c r="L21" s="66" t="n"/>
+      <c r="L21" s="46" t="inlineStr">
+        <is>
+          <t>검수자
+판정</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="24" customHeight="1" s="49">
       <c r="C22" s="69" t="n"/>
@@ -3197,98 +3260,98 @@
       <c r="K27" s="42" t="n"/>
       <c r="L27" s="66" t="n"/>
     </row>
-    <row r="28" ht="27.75" customHeight="1" s="49">
-      <c r="C28" s="46" t="n"/>
-      <c r="D28" s="46" t="n"/>
-      <c r="E28" s="46" t="n"/>
-      <c r="F28" s="46" t="n"/>
-      <c r="G28" s="46" t="n"/>
-      <c r="H28" s="46" t="n"/>
-      <c r="I28" s="46" t="n"/>
-      <c r="J28" s="46" t="n"/>
-      <c r="K28" s="46" t="n"/>
-      <c r="L28" s="46" t="n"/>
-    </row>
-    <row r="29" ht="19.5" customHeight="1" s="49">
-      <c r="C29" s="121" t="inlineStr">
+    <row r="28" ht="24" customHeight="1" s="49">
+      <c r="C28" s="69" t="n"/>
+      <c r="D28" s="55" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="41" t="n"/>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="47" t="n"/>
+      <c r="J28" s="44" t="n"/>
+      <c r="K28" s="42" t="n"/>
+      <c r="L28" s="66" t="n"/>
+    </row>
+    <row r="29" ht="27.75" customHeight="1" s="49">
+      <c r="C29" s="46" t="n"/>
+      <c r="D29" s="46" t="n"/>
+      <c r="E29" s="46" t="n"/>
+      <c r="F29" s="46" t="n"/>
+      <c r="G29" s="46" t="n"/>
+      <c r="H29" s="46" t="n"/>
+      <c r="I29" s="46" t="n"/>
+      <c r="J29" s="46" t="n"/>
+      <c r="K29" s="46" t="n"/>
+      <c r="L29" s="46" t="n"/>
+    </row>
+    <row r="30" ht="19.5" customHeight="1" s="49">
+      <c r="C30" s="121" t="inlineStr">
         <is>
           <t>3. 이슈 및 지원요청  —  대안 없이 문제만 올리는 보고는 반려</t>
         </is>
       </c>
-      <c r="D29" s="64" t="n"/>
-      <c r="E29" s="64" t="n"/>
-      <c r="F29" s="64" t="n"/>
-      <c r="G29" s="64" t="n"/>
-      <c r="H29" s="64" t="n"/>
-      <c r="I29" s="64" t="n"/>
-      <c r="J29" s="64" t="n"/>
-      <c r="K29" s="64" t="n"/>
-      <c r="L29" s="65" t="n"/>
-    </row>
-    <row r="30" ht="27.75" customHeight="1" s="49">
-      <c r="C30" s="46" t="inlineStr">
+      <c r="D30" s="64" t="n"/>
+      <c r="E30" s="64" t="n"/>
+      <c r="F30" s="64" t="n"/>
+      <c r="G30" s="64" t="n"/>
+      <c r="H30" s="64" t="n"/>
+      <c r="I30" s="64" t="n"/>
+      <c r="J30" s="64" t="n"/>
+      <c r="K30" s="64" t="n"/>
+      <c r="L30" s="65" t="n"/>
+    </row>
+    <row r="31" ht="27.75" customHeight="1" s="49">
+      <c r="C31" s="46" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="D30" s="46" t="inlineStr">
+      <c r="D31" s="46" t="inlineStr">
         <is>
           <t>이슈 내용</t>
         </is>
       </c>
-      <c r="E30" s="46" t="inlineStr">
+      <c r="E31" s="46" t="inlineStr">
         <is>
           <t>영향
 (일정/비용/품질)</t>
         </is>
       </c>
-      <c r="F30" s="46" t="inlineStr">
+      <c r="F31" s="46" t="inlineStr">
         <is>
           <t>근본 원인</t>
         </is>
       </c>
-      <c r="G30" s="46" t="inlineStr">
+      <c r="G31" s="46" t="inlineStr">
         <is>
           <t>대안 1</t>
         </is>
       </c>
-      <c r="H30" s="46" t="inlineStr">
+      <c r="H31" s="46" t="inlineStr">
         <is>
           <t>대안 2</t>
         </is>
       </c>
-      <c r="I30" s="46" t="inlineStr">
+      <c r="I31" s="46" t="inlineStr">
         <is>
           <t>권고안</t>
         </is>
       </c>
-      <c r="J30" s="46" t="inlineStr">
+      <c r="J31" s="46" t="inlineStr">
         <is>
           <t>요청사항</t>
         </is>
       </c>
-      <c r="K30" s="46" t="inlineStr">
+      <c r="K31" s="46" t="inlineStr">
         <is>
           <t>결정기한</t>
         </is>
       </c>
-      <c r="L30" s="46" t="inlineStr">
+      <c r="L31" s="46" t="inlineStr">
         <is>
           <t>대표 결정</t>
         </is>
       </c>
-    </row>
-    <row r="31" ht="36" customHeight="1" s="49">
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="18" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="18" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="18" t="n"/>
-      <c r="I31" s="18" t="n"/>
-      <c r="J31" s="18" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="66" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1" s="49">
       <c r="C32" s="6" t="n"/>
@@ -3314,104 +3377,102 @@
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="66" t="n"/>
     </row>
-    <row r="34" ht="27.75" customHeight="1" s="49">
-      <c r="C34" s="13" t="n"/>
-      <c r="D34" s="46" t="n"/>
-      <c r="E34" s="46" t="n"/>
-      <c r="F34" s="46" t="n"/>
-      <c r="G34" s="46" t="n"/>
-      <c r="H34" s="46" t="n"/>
-      <c r="I34" s="46" t="n"/>
-      <c r="J34" s="46" t="n"/>
-      <c r="K34" s="46" t="n"/>
-      <c r="L34" s="46" t="n"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1" s="49">
-      <c r="C35" s="121" t="inlineStr">
+    <row r="34" ht="36" customHeight="1" s="49">
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="18" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="18" t="n"/>
+      <c r="G34" s="18" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="18" t="n"/>
+      <c r="J34" s="18" t="n"/>
+      <c r="K34" s="6" t="n"/>
+      <c r="L34" s="66" t="n"/>
+    </row>
+    <row r="35" ht="27.75" customHeight="1" s="49">
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="46" t="n"/>
+      <c r="E35" s="46" t="n"/>
+      <c r="F35" s="46" t="n"/>
+      <c r="G35" s="46" t="n"/>
+      <c r="H35" s="46" t="n"/>
+      <c r="I35" s="46" t="n"/>
+      <c r="J35" s="46" t="n"/>
+      <c r="K35" s="46" t="n"/>
+      <c r="L35" s="46" t="n"/>
+    </row>
+    <row r="36" ht="19.5" customHeight="1" s="49">
+      <c r="C36" s="121" t="inlineStr">
         <is>
           <t>4. 다음 주 제안 업무  —  지시를 기다리지 말 것. 본인이 먼저 제안.</t>
         </is>
       </c>
-      <c r="D35" s="64" t="n"/>
-      <c r="E35" s="64" t="n"/>
-      <c r="F35" s="64" t="n"/>
-      <c r="G35" s="64" t="n"/>
-      <c r="H35" s="64" t="n"/>
-      <c r="I35" s="64" t="n"/>
-      <c r="J35" s="64" t="n"/>
-      <c r="K35" s="64" t="n"/>
-      <c r="L35" s="65" t="n"/>
-    </row>
-    <row r="36" ht="27.75" customHeight="1" s="49">
-      <c r="C36" s="13" t="inlineStr">
+      <c r="D36" s="64" t="n"/>
+      <c r="E36" s="64" t="n"/>
+      <c r="F36" s="64" t="n"/>
+      <c r="G36" s="64" t="n"/>
+      <c r="H36" s="64" t="n"/>
+      <c r="I36" s="64" t="n"/>
+      <c r="J36" s="64" t="n"/>
+      <c r="K36" s="64" t="n"/>
+      <c r="L36" s="65" t="n"/>
+    </row>
+    <row r="37" ht="27.75" customHeight="1" s="49">
+      <c r="C37" s="13" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D36" s="46" t="inlineStr">
+      <c r="D37" s="46" t="inlineStr">
         <is>
           <t>제안 업무</t>
         </is>
       </c>
-      <c r="E36" s="46" t="inlineStr">
+      <c r="E37" s="46" t="inlineStr">
         <is>
           <t>왜 해야 하는가</t>
         </is>
       </c>
-      <c r="F36" s="46" t="inlineStr">
+      <c r="F37" s="46" t="inlineStr">
         <is>
           <t>완료기준(안)</t>
         </is>
       </c>
-      <c r="G36" s="46" t="inlineStr">
+      <c r="G37" s="46" t="inlineStr">
         <is>
           <t>예상
 소요(h)</t>
         </is>
       </c>
-      <c r="H36" s="46" t="inlineStr">
+      <c r="H37" s="46" t="inlineStr">
         <is>
           <t>우선순위(안)</t>
         </is>
       </c>
-      <c r="I36" s="46" t="inlineStr">
+      <c r="I37" s="46" t="inlineStr">
         <is>
           <t>선행 조건</t>
         </is>
       </c>
-      <c r="J36" s="46" t="inlineStr">
+      <c r="J37" s="46" t="inlineStr">
         <is>
           <t>필요 지원</t>
         </is>
       </c>
-      <c r="K36" s="46" t="inlineStr">
+      <c r="K37" s="46" t="inlineStr">
         <is>
           <t>대표 승인</t>
         </is>
       </c>
-      <c r="L36" s="46" t="inlineStr">
+      <c r="L37" s="46" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
-    </row>
-    <row r="37" ht="31.5" customHeight="1" s="49">
-      <c r="C37" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="18" t="n"/>
-      <c r="E37" s="18" t="n"/>
-      <c r="F37" s="18" t="n"/>
-      <c r="G37" s="114" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="18" t="n"/>
-      <c r="J37" s="18" t="n"/>
-      <c r="K37" s="66" t="n"/>
-      <c r="L37" s="6" t="n"/>
     </row>
     <row r="38" ht="31.5" customHeight="1" s="49">
       <c r="C38" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="18" t="n"/>
       <c r="E38" s="18" t="n"/>
@@ -3425,7 +3486,7 @@
     </row>
     <row r="39" ht="31.5" customHeight="1" s="49">
       <c r="C39" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D39" s="18" t="n"/>
       <c r="E39" s="18" t="n"/>
@@ -3439,7 +3500,7 @@
     </row>
     <row r="40" ht="31.5" customHeight="1" s="49">
       <c r="C40" s="22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40" s="18" t="n"/>
       <c r="E40" s="18" t="n"/>
@@ -3451,51 +3512,41 @@
       <c r="K40" s="66" t="n"/>
       <c r="L40" s="6" t="n"/>
     </row>
-    <row r="41" ht="25.5" customHeight="1" s="49">
-      <c r="C41" s="45" t="n"/>
-      <c r="D41" s="43" t="n"/>
-      <c r="J41" s="58" t="n"/>
-    </row>
-    <row r="42" ht="19.5" customHeight="1" s="49">
-      <c r="C42" s="48" t="inlineStr">
+    <row r="41" ht="31.5" customHeight="1" s="49">
+      <c r="C41" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" s="18" t="n"/>
+      <c r="E41" s="18" t="n"/>
+      <c r="F41" s="18" t="n"/>
+      <c r="G41" s="114" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="18" t="n"/>
+      <c r="J41" s="18" t="n"/>
+      <c r="K41" s="66" t="n"/>
+      <c r="L41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="25.5" customHeight="1" s="49">
+      <c r="C42" s="45" t="n"/>
+      <c r="D42" s="43" t="n"/>
+      <c r="J42" s="58" t="n"/>
+    </row>
+    <row r="43" ht="19.5" customHeight="1" s="49">
+      <c r="C43" s="48" t="inlineStr">
         <is>
           <t>5. 자기점검 및 대표 검수</t>
         </is>
       </c>
-    </row>
-    <row r="43" ht="25.5" customHeight="1" s="49">
-      <c r="C43" s="45" t="inlineStr">
-        <is>
-          <t>이번 주 가장 잘한 것</t>
-        </is>
-      </c>
-      <c r="D43" s="43" t="inlineStr">
-        <is>
-          <t>결과로 증명되는 것 1개만</t>
-        </is>
-      </c>
-      <c r="E43" s="41" t="n"/>
-      <c r="F43" s="41" t="n"/>
-      <c r="G43" s="41" t="n"/>
-      <c r="H43" s="41" t="n"/>
-      <c r="I43" s="42" t="n"/>
-      <c r="J43" s="58" t="inlineStr">
-        <is>
-          <t>[대표 검수 의견]</t>
-        </is>
-      </c>
-      <c r="K43" s="59" t="n"/>
-      <c r="L43" s="60" t="n"/>
     </row>
     <row r="44" ht="25.5" customHeight="1" s="49">
       <c r="C44" s="45" t="inlineStr">
         <is>
-          <t>이번 주 가장 부족한 것</t>
+          <t>이번 주 가장 잘한 것</t>
         </is>
       </c>
       <c r="D44" s="43" t="inlineStr">
         <is>
-          <t>변명 말고 사실만</t>
+          <t>결과로 증명되는 것 1개만</t>
         </is>
       </c>
       <c r="E44" s="41" t="n"/>
@@ -3503,18 +3554,23 @@
       <c r="G44" s="41" t="n"/>
       <c r="H44" s="41" t="n"/>
       <c r="I44" s="42" t="n"/>
-      <c r="J44" s="61" t="n"/>
-      <c r="L44" s="62" t="n"/>
+      <c r="J44" s="58" t="inlineStr">
+        <is>
+          <t>[대표 검수 의견]</t>
+        </is>
+      </c>
+      <c r="K44" s="59" t="n"/>
+      <c r="L44" s="60" t="n"/>
     </row>
     <row r="45" ht="25.5" customHeight="1" s="49">
       <c r="C45" s="45" t="inlineStr">
         <is>
-          <t>다음 주 개선 액션 1개</t>
+          <t>이번 주 가장 부족한 것</t>
         </is>
       </c>
       <c r="D45" s="43" t="inlineStr">
         <is>
-          <t>실행 가능한 행동으로</t>
+          <t>변명 말고 사실만</t>
         </is>
       </c>
       <c r="E45" s="41" t="n"/>
@@ -3522,85 +3578,112 @@
       <c r="G45" s="41" t="n"/>
       <c r="H45" s="41" t="n"/>
       <c r="I45" s="42" t="n"/>
-      <c r="J45" s="63" t="n"/>
-      <c r="K45" s="64" t="n"/>
-      <c r="L45" s="65" t="n"/>
+      <c r="J45" s="61" t="n"/>
+      <c r="L45" s="62" t="n"/>
+    </row>
+    <row r="46" ht="25.5" customHeight="1" s="49">
+      <c r="C46" s="45" t="inlineStr">
+        <is>
+          <t>다음 주 개선 액션 1개</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>실행 가능한 행동으로</t>
+        </is>
+      </c>
+      <c r="E46" s="41" t="n"/>
+      <c r="F46" s="41" t="n"/>
+      <c r="G46" s="41" t="n"/>
+      <c r="H46" s="41" t="n"/>
+      <c r="I46" s="42" t="n"/>
+      <c r="J46" s="63" t="n"/>
+      <c r="K46" s="64" t="n"/>
+      <c r="L46" s="65" t="n"/>
     </row>
     <row r="47" ht="33.75" customHeight="1" s="49">
-      <c r="C47" s="45" t="inlineStr">
+      <c r="C47" s="45" t="n"/>
+      <c r="D47" s="47" t="n"/>
+      <c r="G47" s="45" t="n"/>
+      <c r="H47" s="66" t="n"/>
+      <c r="J47" s="45" t="n"/>
+      <c r="K47" s="56" t="n"/>
+    </row>
+    <row r="48" ht="33.75" customHeight="1" s="49">
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>제출자</t>
         </is>
       </c>
-      <c r="D47" s="47" t="n"/>
-      <c r="E47" s="41" t="n"/>
-      <c r="F47" s="42" t="n"/>
-      <c r="G47" s="45" t="inlineStr">
+      <c r="D48" s="47" t="n"/>
+      <c r="E48" s="41" t="n"/>
+      <c r="F48" s="42" t="n"/>
+      <c r="G48" s="45" t="inlineStr">
         <is>
           <t>검수자</t>
         </is>
       </c>
-      <c r="H47" s="66" t="n"/>
-      <c r="I47" s="42" t="n"/>
-      <c r="J47" s="45" t="inlineStr">
+      <c r="H48" s="66" t="n"/>
+      <c r="I48" s="42" t="n"/>
+      <c r="J48" s="45" t="inlineStr">
         <is>
           <t>최종 판정</t>
         </is>
       </c>
-      <c r="K47" s="56" t="n"/>
-      <c r="L47" s="42" t="n"/>
+      <c r="K48" s="56" t="n"/>
+      <c r="L48" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D48:F48"/>
+    <mergeCell ref="J28:K28"/>
     <mergeCell ref="D22:H22"/>
-    <mergeCell ref="D47:F47"/>
     <mergeCell ref="D7:L7"/>
-    <mergeCell ref="D43:I43"/>
-    <mergeCell ref="C19:L19"/>
     <mergeCell ref="D21:H21"/>
-    <mergeCell ref="K47:L47"/>
     <mergeCell ref="J24:K24"/>
     <mergeCell ref="D27:H27"/>
+    <mergeCell ref="C30:L30"/>
     <mergeCell ref="J27:K27"/>
-    <mergeCell ref="C42:L42"/>
-    <mergeCell ref="D17:E17"/>
     <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J18:L18"/>
     <mergeCell ref="J25:K25"/>
-    <mergeCell ref="C29:L29"/>
-    <mergeCell ref="C35:L35"/>
-    <mergeCell ref="J43:L45"/>
-    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="D28:H28"/>
+    <mergeCell ref="C20:L20"/>
+    <mergeCell ref="D18:E18"/>
     <mergeCell ref="D44:I44"/>
     <mergeCell ref="J22:K22"/>
-    <mergeCell ref="H47:I47"/>
     <mergeCell ref="C1:L1"/>
+    <mergeCell ref="K48:L48"/>
     <mergeCell ref="J21:K21"/>
     <mergeCell ref="D25:H25"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="D46:I46"/>
     <mergeCell ref="C9:L9"/>
     <mergeCell ref="D24:H24"/>
     <mergeCell ref="D45:I45"/>
     <mergeCell ref="D23:H23"/>
+    <mergeCell ref="C43:L43"/>
+    <mergeCell ref="J44:L46"/>
     <mergeCell ref="J23:K23"/>
     <mergeCell ref="C2:L2"/>
     <mergeCell ref="D6:L6"/>
+    <mergeCell ref="C36:L36"/>
     <mergeCell ref="D26:H26"/>
   </mergeCells>
   <dataValidations count="5">
-    <dataValidation sqref="I21:I27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I22:I28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"충족,미충족"</formula1>
     </dataValidation>
-    <dataValidation sqref="L21:L27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L22:L28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,보완,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="K37:K40 L31:L33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K38:K41 L32:L34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"승인,보류,반려"</formula1>
     </dataValidation>
-    <dataValidation sqref="K47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"합격,조건부합격,보완요청,불합격"</formula1>
     </dataValidation>
-    <dataValidation sqref="G12:G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G12:G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"완료,진행중,미착수,보류,취소"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>